<commit_message>
TASK#10.6: No-Evidence Full Suite
</commit_message>
<xml_diff>
--- a/docs/prompts/tasks/TASK-10-local-stored-judge-experience-ux-follow-up/task-10-full-suite-session-plan.xlsx
+++ b/docs/prompts/tasks/TASK-10-local-stored-judge-experience-ux-follow-up/task-10-full-suite-session-plan.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task 10 Plan" sheetId="1" r:id="Rcfff08d913f9408a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usage Guide" sheetId="2" r:id="R78e3ffa37f524f30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task 10 Plan" sheetId="1" r:id="Rc30c29383ae8433b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usage Guide" sheetId="2" r:id="Rb81cf2bda715459b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -592,15 +592,23 @@
       <x:c r="K4" s="27" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="L4" s="27"/>
-      <x:c r="M4" s="3"/>
-      <x:c r="N4" s="3"/>
-      <x:c r="O4" s="3"/>
+      <x:c r="L4" s="27" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="M4" s="3" t="str">
+        <x:v>2026-07-22 10:18 BRT</x:v>
+      </x:c>
+      <x:c r="N4" s="3" t="str">
+        <x:v>2026-07-22 10:36 BRT</x:v>
+      </x:c>
+      <x:c r="O4" s="3" t="str">
+        <x:v>Pending PR creation</x:v>
+      </x:c>
       <x:c r="P4" s="3" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="Q4" s="8" t="str">
-        <x:v>Fill actuals after the task PR is complete.</x:v>
+        <x:v>Missing evidence is deferred/non-blocking for Task 10.6; outcomes, failed notes, and measurements still block. xcodebuild build and build-for-testing succeeded; xcodebuild test could not run because no concrete simulator was available in the sandbox. Token actuals unavailable in Codex desktop telemetry.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -729,7 +737,7 @@
       </x:c>
       <x:c r="L8" s="28" t="n">
         <x:f>SUM(L2:L6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="M8" s="10"/>
       <x:c r="N8" s="10"/>

</xml_diff>

<commit_message>
Track TASK#10.6 PR URL
</commit_message>
<xml_diff>
--- a/docs/prompts/tasks/TASK-10-local-stored-judge-experience-ux-follow-up/task-10-full-suite-session-plan.xlsx
+++ b/docs/prompts/tasks/TASK-10-local-stored-judge-experience-ux-follow-up/task-10-full-suite-session-plan.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task 10 Plan" sheetId="1" r:id="Rc30c29383ae8433b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usage Guide" sheetId="2" r:id="Rb81cf2bda715459b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task 10 Plan" sheetId="1" r:id="R609ddfe1b3a94ac6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usage Guide" sheetId="2" r:id="Ra0c963013ff34e53"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -602,10 +602,10 @@
         <x:v>2026-07-22 10:36 BRT</x:v>
       </x:c>
       <x:c r="O4" s="3" t="str">
-        <x:v>Pending PR creation</x:v>
+        <x:v>https://github.com/diegomhamilton/fsae-competition-app/pull/82</x:v>
       </x:c>
       <x:c r="P4" s="3" t="str">
-        <x:v>Implemented</x:v>
+        <x:v>PR Opened</x:v>
       </x:c>
       <x:c r="Q4" s="8" t="str">
         <x:v>Missing evidence is deferred/non-blocking for Task 10.6; outcomes, failed notes, and measurements still block. xcodebuild build and build-for-testing succeeded; xcodebuild test could not run because no concrete simulator was available in the sandbox. Token actuals unavailable in Codex desktop telemetry.</x:v>

</xml_diff>

<commit_message>
TASK#10.6: No-Evidence Full Suite (#82)
* TASK#10.6: No-Evidence Full Suite

* Track TASK#10.6 PR URL

* TASK#11: polish inspection flow UI

* TASK#10.6: disable team switching
</commit_message>
<xml_diff>
--- a/docs/prompts/tasks/TASK-10-local-stored-judge-experience-ux-follow-up/task-10-full-suite-session-plan.xlsx
+++ b/docs/prompts/tasks/TASK-10-local-stored-judge-experience-ux-follow-up/task-10-full-suite-session-plan.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task 10 Plan" sheetId="1" r:id="Rcfff08d913f9408a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usage Guide" sheetId="2" r:id="R78e3ffa37f524f30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task 10 Plan" sheetId="1" r:id="R609ddfe1b3a94ac6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usage Guide" sheetId="2" r:id="Ra0c963013ff34e53"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -592,15 +592,23 @@
       <x:c r="K4" s="27" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="L4" s="27"/>
-      <x:c r="M4" s="3"/>
-      <x:c r="N4" s="3"/>
-      <x:c r="O4" s="3"/>
+      <x:c r="L4" s="27" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="M4" s="3" t="str">
+        <x:v>2026-07-22 10:18 BRT</x:v>
+      </x:c>
+      <x:c r="N4" s="3" t="str">
+        <x:v>2026-07-22 10:36 BRT</x:v>
+      </x:c>
+      <x:c r="O4" s="3" t="str">
+        <x:v>https://github.com/diegomhamilton/fsae-competition-app/pull/82</x:v>
+      </x:c>
       <x:c r="P4" s="3" t="str">
-        <x:v>Planned</x:v>
+        <x:v>PR Opened</x:v>
       </x:c>
       <x:c r="Q4" s="8" t="str">
-        <x:v>Fill actuals after the task PR is complete.</x:v>
+        <x:v>Missing evidence is deferred/non-blocking for Task 10.6; outcomes, failed notes, and measurements still block. xcodebuild build and build-for-testing succeeded; xcodebuild test could not run because no concrete simulator was available in the sandbox. Token actuals unavailable in Codex desktop telemetry.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -729,7 +737,7 @@
       </x:c>
       <x:c r="L8" s="28" t="n">
         <x:f>SUM(L2:L6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="M8" s="10"/>
       <x:c r="N8" s="10"/>

</xml_diff>

<commit_message>
TASK#10.7: Update tracking workbook
</commit_message>
<xml_diff>
--- a/docs/prompts/tasks/TASK-10-local-stored-judge-experience-ux-follow-up/task-10-full-suite-session-plan.xlsx
+++ b/docs/prompts/tasks/TASK-10-local-stored-judge-experience-ux-follow-up/task-10-full-suite-session-plan.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task 10 Plan" sheetId="1" r:id="R609ddfe1b3a94ac6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usage Guide" sheetId="2" r:id="Ra0c963013ff34e53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task 10 Plan" sheetId="1" r:id="Rc4631dcb8ca141a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usage Guide" sheetId="2" r:id="Rc53a2c3a771f47b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -622,7 +622,7 @@
         <x:v>Confirmed reset, preserved completed executions, and past session start/end timestamp review.</x:v>
       </x:c>
       <x:c r="D5" s="3" t="str">
-        <x:v>codex/task-10-7-reset-and-history</x:v>
+        <x:v>task_10-7_switch_sessions</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
         <x:v>gpt-5.6-sol</x:v>
@@ -641,15 +641,23 @@
       <x:c r="K5" s="27" t="n">
         <x:v>8.5</x:v>
       </x:c>
-      <x:c r="L5" s="27"/>
-      <x:c r="M5" s="3"/>
-      <x:c r="N5" s="3"/>
-      <x:c r="O5" s="3"/>
+      <x:c r="L5" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M5" s="3" t="str">
+        <x:v>2026-08-21 09:34 BRT</x:v>
+      </x:c>
+      <x:c r="N5" s="3" t="str">
+        <x:v>2026-08-21 10:34 BRT</x:v>
+      </x:c>
+      <x:c r="O5" s="3" t="str">
+        <x:v>https://github.com/diegomhamilton/fsae-competition-app/pull/85</x:v>
+      </x:c>
       <x:c r="P5" s="3" t="str">
-        <x:v>Planned</x:v>
+        <x:v>PR Opened</x:v>
       </x:c>
       <x:c r="Q5" s="8" t="str">
-        <x:v>Fill actuals after the task PR is complete.</x:v>
+        <x:v>Confirmed reset clears only the active draft directory and session catalog record; submitted snapshots and completed session records remain. Read-only past executions show start/end timestamps and an explicit empty state. xcodebuild build-for-testing succeeded (exit 0); targeted simulator execution could not be finalized in the current approval environment. Token actuals unavailable in Codex desktop telemetry.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -737,7 +745,7 @@
       </x:c>
       <x:c r="L8" s="28" t="n">
         <x:f>SUM(L2:L6)</x:f>
-        <x:v>1.25</x:v>
+        <x:v>2.25</x:v>
       </x:c>
       <x:c r="M8" s="10"/>
       <x:c r="N8" s="10"/>

</xml_diff>